<commit_message>
Datos Excel y word
</commit_message>
<xml_diff>
--- a/Docs/ISIS1225 - Tablas de Datos Lab 5.xlsx
+++ b/Docs/ISIS1225 - Tablas de Datos Lab 5.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Lina/Library/Mobile Documents/com~apple~CloudDocs/Universidad/EDA/ISIS1225-Laboratorio-5/Docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/206f61cbe57f6cb9/Desktop/EDA/ISIS1225-Laboratorio-5-G06/Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{956D6578-0A0A-6148-A156-5D7CA8FF2F1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{956D6578-0A0A-6148-A156-5D7CA8FF2F1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{141E2B03-C8A4-4655-898F-CA6EE41FCE8A}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17580" xr2:uid="{D82936D8-D2C9-4EB2-9CBC-3665F65B95FD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="8" xr2:uid="{D82936D8-D2C9-4EB2-9CBC-3665F65B95FD}"/>
   </bookViews>
   <sheets>
     <sheet name="01-Data" sheetId="1" r:id="rId1"/>
@@ -55,10 +55,10 @@
     <t>Tamaño de la muestra (LINKED_LIST)</t>
   </si>
   <si>
-    <t xml:space="preserve">Algoritmo iterativo (especificar) </t>
+    <t xml:space="preserve">Algoritmo iterativo (Shell Sort) </t>
   </si>
   <si>
-    <t>Algoritmo recursivo (especificar)</t>
+    <t>Algoritmo recursivo (Merge Sort)</t>
   </si>
   <si>
     <t>TIEMPOS DE EJECUCIÓN MEJORES ALGORITMOS [ms]</t>
@@ -465,6 +465,85 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Dax-Regular"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Dax-Regular"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Dax-Regular"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <strike val="0"/>
@@ -580,85 +659,6 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Dax-Regular"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Dax-Regular"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Dax-Regular"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1055,7 +1055,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1209,6 +1209,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.42</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>37.9</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>164.7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>691.42</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1521.43</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6812.23</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>22364.240000000002</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>25151.83</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1296,6 +1320,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.68</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46.4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>188.19</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>760.91</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1711.17</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4905.1400000000003</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>13371.13</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>22654.59</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1383,6 +1431,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.19</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.53</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>11.75</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>35.369999999999997</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>72.02</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>187.35</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>432.32</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>631.94000000000005</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1470,6 +1542,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.24</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.72</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.83</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>13.9</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20.46</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>37.94</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>58.64</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>75.319999999999993</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1557,6 +1653,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.34</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.62</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9.99</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>26.4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>53.48</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>116.21</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>297.77999999999997</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>391.95</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1857,6 +1977,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1864,7 +1985,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1897,7 +2017,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2051,6 +2171,18 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>4.33</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2965.24</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>24754.34</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>202321.73</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2138,6 +2270,18 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>3.8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3381.2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>38877.99</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>362774.97</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2225,6 +2369,24 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>2.0299999999999998</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>434.31</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2359.62</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>27320.11</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>78028.06</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>254006.03</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2312,6 +2474,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.51</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20.84</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>73.489999999999995</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>301.97000000000003</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>705.43</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1878.21</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4866.72</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9361.26</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2399,6 +2585,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1.1000000000000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>38.39</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>252.06</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>867.92</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1555.2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5260.82</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>15920.2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>65943.460000000006</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2700,6 +2910,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2707,7 +2918,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2740,7 +2950,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2855,6 +3065,50 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>'01-Data'!$A$3:$A$10</c:f>
@@ -2894,6 +3148,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.42</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>37.9</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>164.7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>691.42</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1521.43</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6812.23</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>22364.240000000002</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>25151.83</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2942,6 +3220,50 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>'01-Data'!$A$14:$A$21</c:f>
@@ -2981,6 +3303,18 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>4.33</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2965.24</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>24754.34</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>202321.73</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -3282,6 +3616,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3289,7 +3624,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3322,7 +3656,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -3437,6 +3771,50 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>'01-Data'!$A$3:$A$10</c:f>
@@ -3476,6 +3854,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.68</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46.4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>188.19</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>760.91</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1711.17</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4905.1400000000003</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>13371.13</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>22654.59</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -3524,6 +3926,50 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>'01-Data'!$A$14:$A$21</c:f>
@@ -3563,6 +4009,18 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>3.8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3381.2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>38877.99</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>362774.97</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -3864,6 +4322,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3871,7 +4330,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3904,7 +4362,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -4019,6 +4477,50 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>'01-Data'!$A$3:$A$10</c:f>
@@ -4058,6 +4560,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.19</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.53</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>11.75</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>35.369999999999997</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>72.02</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>187.35</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>432.32</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>631.94000000000005</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -4106,6 +4632,50 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>'01-Data'!$A$14:$A$21</c:f>
@@ -4145,6 +4715,24 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>2.0299999999999998</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>434.31</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2359.62</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>27320.11</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>78028.06</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>254006.03</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -4446,6 +5034,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -4453,7 +5042,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4486,7 +5074,7 @@
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -4601,6 +5189,50 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>'01-Data'!$A$3:$A$10</c:f>
@@ -4640,6 +5272,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.24</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.72</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.83</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>13.9</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20.46</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>37.94</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>58.64</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>75.319999999999993</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -4688,6 +5344,50 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>'01-Data'!$A$14:$A$21</c:f>
@@ -4727,6 +5427,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.51</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20.84</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>73.489999999999995</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>301.97000000000003</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>705.43</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1878.21</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4866.72</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9361.26</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -5028,6 +5752,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -5035,7 +5760,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -5068,7 +5792,7 @@
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -5178,6 +5902,50 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>'01-Data'!$A$3:$A$10</c:f>
@@ -5217,6 +5985,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.34</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.62</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9.99</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>26.4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>53.48</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>116.21</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>297.77999999999997</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>391.95</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -5265,6 +6057,50 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>'01-Data'!$A$14:$A$21</c:f>
@@ -5304,6 +6140,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1.1000000000000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>38.39</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>252.06</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>867.92</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1555.2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5260.82</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>15920.2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>65943.460000000006</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -5605,6 +6465,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -5612,7 +6473,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -5645,7 +6505,7 @@
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -5731,7 +6591,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Algoritmo iterativo (especificar) </c:v>
+                  <c:v>Algoritmo iterativo (Shell Sort) </c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5760,6 +6620,50 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>'01-Data'!$A$25:$A$32</c:f>
@@ -5799,6 +6703,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.19</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.53</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>11.75</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>35.369999999999997</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>72.02</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>187.35</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>432.32</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>631.94000000000005</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -5818,7 +6746,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Algoritmo recursivo (especificar)</c:v>
+                  <c:v>Algoritmo recursivo (Merge Sort)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5847,6 +6775,50 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>'01-Data'!$A$25:$A$32</c:f>
@@ -5886,6 +6858,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.24</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.72</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.83</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>13.9</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20.46</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>37.94</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>58.64</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>75.319999999999993</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -6187,6 +7183,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -6194,7 +7191,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10756,7 +11752,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8676640" cy="6289040"/>
+    <xdr:ext cx="8656320" cy="6278880"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Gráfico 1">
@@ -10822,7 +11818,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8674100" cy="6286500"/>
+    <xdr:ext cx="8656320" cy="6278880"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Gráfico 1">
@@ -10855,7 +11851,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8674100" cy="6286500"/>
+    <xdr:ext cx="8656320" cy="6278880"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Gráfico 1">
@@ -10888,7 +11884,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8674100" cy="6286500"/>
+    <xdr:ext cx="8656320" cy="6278880"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Gráfico 1">
@@ -10921,7 +11917,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8674100" cy="6286500"/>
+    <xdr:ext cx="8656320" cy="6278880"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -10954,7 +11950,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8674100" cy="6286500"/>
+    <xdr:ext cx="8656320" cy="6278880"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -10987,7 +11983,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8674100" cy="6286500"/>
+    <xdr:ext cx="8656320" cy="6278880"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Gráfico 1">
@@ -11058,18 +12054,18 @@
     <tableColumn id="2" xr3:uid="{4F9B7329-040C-4D35-96E7-B9181424DC65}" name="Tamaño de la muestra (LINKED_LIST)" dataDxfId="12">
       <calculatedColumnFormula>Table13[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BDA028DF-4CED-4928-B040-96AD8F8A43EB}" name="Insertion Sort Linked List" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{A5E99D51-DD73-48A7-AE0D-601A8EE89AFA}" name="Selection Sort Linked List" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{A2E3ADDC-6DD2-4948-B1D7-3CE7770DFC65}" name="Shell Sort Linked List" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{CE9F6C54-1CFA-E54C-8FB6-7838A5EDD8A3}" name="Merge Sort Linked List" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{B636EE2A-F13E-2342-B329-EE5C61F78A76}" name="Quick Sort Linked List" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{BDA028DF-4CED-4928-B040-96AD8F8A43EB}" name="Insertion Sort Linked List" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{A5E99D51-DD73-48A7-AE0D-601A8EE89AFA}" name="Selection Sort Linked List" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{A2E3ADDC-6DD2-4948-B1D7-3CE7770DFC65}" name="Shell Sort Linked List" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{CE9F6C54-1CFA-E54C-8FB6-7838A5EDD8A3}" name="Merge Sort Linked List" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{B636EE2A-F13E-2342-B329-EE5C61F78A76}" name="Quick Sort Linked List" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4009FC45-711A-7E4A-BD3C-BEB6C9914449}" name="Tabla3" displayName="Tabla3" ref="A24:D32" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4009FC45-711A-7E4A-BD3C-BEB6C9914449}" name="Tabla3" displayName="Tabla3" ref="A24:D32" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="5" tableBorderDxfId="4">
   <autoFilter ref="A24:D32" xr:uid="{4009FC45-711A-7E4A-BD3C-BEB6C9914449}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -11077,19 +12073,19 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{B41C1FDF-31EB-8245-9B27-55998E13A758}" name="Porcentaje de la muestra [pct]" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{A5516E25-E137-844A-8ACE-E872C6D3AF26}" name="Tamaño de la muestra " dataDxfId="7">
+    <tableColumn id="1" xr3:uid="{B41C1FDF-31EB-8245-9B27-55998E13A758}" name="Porcentaje de la muestra [pct]" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{A5516E25-E137-844A-8ACE-E872C6D3AF26}" name="Tamaño de la muestra " dataDxfId="2">
       <calculatedColumnFormula>Tabla3[[#This Row],[Porcentaje de la muestra '[pct']]] *10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{FCABA3BF-6045-0E48-BB37-6E396D6328EB}" name="Algoritmo iterativo (especificar) " dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{D7C2D6B9-4643-7546-86E6-D34E7A0D57D5}" name="Algoritmo recursivo (especificar)" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{FCABA3BF-6045-0E48-BB37-6E396D6328EB}" name="Algoritmo iterativo (Shell Sort) " dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{D7C2D6B9-4643-7546-86E6-D34E7A0D57D5}" name="Algoritmo recursivo (Merge Sort)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -11389,14 +12385,14 @@
     <tabColor theme="2" tint="-9.9978637043366805E-2"/>
   </sheetPr>
   <dimension ref="A1:H32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="45.5" style="1" customWidth="1"/>
+    <col min="1" max="1" width="28.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="45.44140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="30.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="31.1640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="24.5" style="3" customWidth="1"/>
-    <col min="6" max="11" width="24.5" customWidth="1"/>
+    <col min="4" max="4" width="31.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="24.44140625" style="3" customWidth="1"/>
+    <col min="6" max="11" width="24.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.25" customHeight="1">
@@ -11410,7 +12406,7 @@
       <c r="F1" s="35"/>
       <c r="G1" s="35"/>
     </row>
-    <row r="2" spans="1:8" s="2" customFormat="1" ht="17" thickBot="1">
+    <row r="2" spans="1:8" s="2" customFormat="1" ht="28.2" thickBot="1">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
@@ -11433,7 +12429,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" s="2" customFormat="1">
+    <row r="3" spans="1:8" s="2" customFormat="1" ht="13.8">
       <c r="A3" s="26">
         <v>5.0000000000000001E-3</v>
       </c>
@@ -11441,13 +12437,23 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>50</v>
       </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="23"/>
+      <c r="C3" s="28">
+        <v>0.42</v>
+      </c>
+      <c r="D3" s="28">
+        <v>0.68</v>
+      </c>
+      <c r="E3" s="29">
+        <v>0.19</v>
+      </c>
+      <c r="F3" s="29">
+        <v>0.24</v>
+      </c>
+      <c r="G3" s="23">
+        <v>0.34</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" s="2" customFormat="1">
+    <row r="4" spans="1:8" s="2" customFormat="1" ht="13.8">
       <c r="A4" s="7">
         <v>0.05</v>
       </c>
@@ -11455,11 +12461,21 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>500</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="13"/>
+      <c r="C4" s="22">
+        <v>37.9</v>
+      </c>
+      <c r="D4" s="22">
+        <v>46.4</v>
+      </c>
+      <c r="E4" s="20">
+        <v>4.53</v>
+      </c>
+      <c r="F4" s="20">
+        <v>2.72</v>
+      </c>
+      <c r="G4" s="13">
+        <v>3.62</v>
+      </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="7">
@@ -11469,11 +12485,21 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>1000</v>
       </c>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="13"/>
+      <c r="C5" s="22">
+        <v>164.7</v>
+      </c>
+      <c r="D5" s="22">
+        <v>188.19</v>
+      </c>
+      <c r="E5" s="20">
+        <v>11.75</v>
+      </c>
+      <c r="F5" s="20">
+        <v>5.83</v>
+      </c>
+      <c r="G5" s="13">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="7">
@@ -11483,11 +12509,21 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>2000</v>
       </c>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="13"/>
+      <c r="C6" s="22">
+        <v>691.42</v>
+      </c>
+      <c r="D6" s="22">
+        <v>760.91</v>
+      </c>
+      <c r="E6" s="20">
+        <v>35.369999999999997</v>
+      </c>
+      <c r="F6" s="20">
+        <v>13.9</v>
+      </c>
+      <c r="G6" s="13">
+        <v>26.4</v>
+      </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="7">
@@ -11497,11 +12533,21 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>3000</v>
       </c>
-      <c r="C7" s="22"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="13"/>
+      <c r="C7" s="22">
+        <v>1521.43</v>
+      </c>
+      <c r="D7" s="22">
+        <v>1711.17</v>
+      </c>
+      <c r="E7" s="20">
+        <v>72.02</v>
+      </c>
+      <c r="F7" s="20">
+        <v>20.46</v>
+      </c>
+      <c r="G7" s="13">
+        <v>53.48</v>
+      </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="7">
@@ -11511,11 +12557,21 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>5000</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="13"/>
+      <c r="C8" s="22">
+        <v>6812.23</v>
+      </c>
+      <c r="D8" s="22">
+        <v>4905.1400000000003</v>
+      </c>
+      <c r="E8" s="20">
+        <v>187.35</v>
+      </c>
+      <c r="F8" s="20">
+        <v>37.94</v>
+      </c>
+      <c r="G8" s="13">
+        <v>116.21</v>
+      </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="7">
@@ -11525,13 +12581,23 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>8000</v>
       </c>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="13"/>
+      <c r="C9" s="22">
+        <v>22364.240000000002</v>
+      </c>
+      <c r="D9" s="22">
+        <v>13371.13</v>
+      </c>
+      <c r="E9" s="20">
+        <v>432.32</v>
+      </c>
+      <c r="F9" s="20">
+        <v>58.64</v>
+      </c>
+      <c r="G9" s="13">
+        <v>297.77999999999997</v>
+      </c>
     </row>
-    <row r="10" spans="1:8" ht="16" thickBot="1">
+    <row r="10" spans="1:8" ht="15" thickBot="1">
       <c r="A10" s="9">
         <v>1</v>
       </c>
@@ -11539,11 +12605,21 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>10000</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="14"/>
+      <c r="C10" s="24">
+        <v>25151.83</v>
+      </c>
+      <c r="D10" s="24">
+        <v>22654.59</v>
+      </c>
+      <c r="E10" s="25">
+        <v>631.94000000000005</v>
+      </c>
+      <c r="F10" s="25">
+        <v>75.319999999999993</v>
+      </c>
+      <c r="G10" s="14">
+        <v>391.95</v>
+      </c>
     </row>
     <row r="11" spans="1:8">
       <c r="E11"/>
@@ -11560,7 +12636,7 @@
       <c r="G12" s="37"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" s="2" customFormat="1" ht="17" thickBot="1">
+    <row r="13" spans="1:8" s="2" customFormat="1" ht="28.2" thickBot="1">
       <c r="A13" s="15" t="s">
         <v>0</v>
       </c>
@@ -11584,7 +12660,7 @@
       </c>
       <c r="H13" s="4"/>
     </row>
-    <row r="14" spans="1:8" s="2" customFormat="1">
+    <row r="14" spans="1:8" s="2" customFormat="1" ht="13.8">
       <c r="A14" s="7">
         <v>5.0000000000000001E-3</v>
       </c>
@@ -11592,14 +12668,24 @@
         <f>Table13[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>50</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="13"/>
+      <c r="C14" s="22">
+        <v>4.33</v>
+      </c>
+      <c r="D14" s="22">
+        <v>3.8</v>
+      </c>
+      <c r="E14" s="22">
+        <v>2.0299999999999998</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0.51</v>
+      </c>
+      <c r="G14" s="13">
+        <v>1.1000000000000001</v>
+      </c>
       <c r="H14" s="8"/>
     </row>
-    <row r="15" spans="1:8" s="2" customFormat="1">
+    <row r="15" spans="1:8" s="2" customFormat="1" ht="13.8">
       <c r="A15" s="7">
         <v>0.05</v>
       </c>
@@ -11607,11 +12693,21 @@
         <f>Table13[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>500</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="13"/>
+      <c r="C15" s="22">
+        <v>2965.24</v>
+      </c>
+      <c r="D15" s="22">
+        <v>3381.2</v>
+      </c>
+      <c r="E15" s="22">
+        <v>434.31</v>
+      </c>
+      <c r="F15" s="4">
+        <v>20.84</v>
+      </c>
+      <c r="G15" s="13">
+        <v>38.39</v>
+      </c>
       <c r="H15" s="8"/>
     </row>
     <row r="16" spans="1:8">
@@ -11622,11 +12718,21 @@
         <f>Table13[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>1000</v>
       </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="13"/>
+      <c r="C16" s="22">
+        <v>24754.34</v>
+      </c>
+      <c r="D16" s="22">
+        <v>38877.99</v>
+      </c>
+      <c r="E16" s="22">
+        <v>2359.62</v>
+      </c>
+      <c r="F16" s="4">
+        <v>73.489999999999995</v>
+      </c>
+      <c r="G16" s="13">
+        <v>252.06</v>
+      </c>
       <c r="H16" s="8"/>
     </row>
     <row r="17" spans="1:8">
@@ -11637,11 +12743,21 @@
         <f>Table13[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>2000</v>
       </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="13"/>
+      <c r="C17" s="22">
+        <v>202321.73</v>
+      </c>
+      <c r="D17" s="22">
+        <v>362774.97</v>
+      </c>
+      <c r="E17" s="22">
+        <v>27320.11</v>
+      </c>
+      <c r="F17" s="4">
+        <v>301.97000000000003</v>
+      </c>
+      <c r="G17" s="13">
+        <v>867.92</v>
+      </c>
       <c r="H17" s="8"/>
     </row>
     <row r="18" spans="1:8">
@@ -11654,9 +12770,15 @@
       </c>
       <c r="C18" s="22"/>
       <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="13"/>
+      <c r="E18" s="22">
+        <v>78028.06</v>
+      </c>
+      <c r="F18" s="4">
+        <v>705.43</v>
+      </c>
+      <c r="G18" s="13">
+        <v>1555.2</v>
+      </c>
       <c r="H18" s="8"/>
     </row>
     <row r="19" spans="1:8">
@@ -11669,9 +12791,15 @@
       </c>
       <c r="C19" s="22"/>
       <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="13"/>
+      <c r="E19" s="22">
+        <v>254006.03</v>
+      </c>
+      <c r="F19" s="4">
+        <v>1878.21</v>
+      </c>
+      <c r="G19" s="13">
+        <v>5260.82</v>
+      </c>
       <c r="H19" s="8"/>
     </row>
     <row r="20" spans="1:8">
@@ -11685,11 +12813,15 @@
       <c r="C20" s="22"/>
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="13"/>
+      <c r="F20" s="4">
+        <v>4866.72</v>
+      </c>
+      <c r="G20" s="13">
+        <v>15920.2</v>
+      </c>
       <c r="H20" s="8"/>
     </row>
-    <row r="21" spans="1:8" ht="16" thickBot="1">
+    <row r="21" spans="1:8" ht="15" thickBot="1">
       <c r="A21" s="9">
         <v>1</v>
       </c>
@@ -11700,11 +12832,15 @@
       <c r="C21" s="24"/>
       <c r="D21" s="24"/>
       <c r="E21" s="24"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="14"/>
+      <c r="F21" s="11">
+        <v>9361.26</v>
+      </c>
+      <c r="G21" s="14">
+        <v>65943.460000000006</v>
+      </c>
       <c r="H21" s="8"/>
     </row>
-    <row r="22" spans="1:8" ht="16" thickBot="1"/>
+    <row r="22" spans="1:8" ht="15" thickBot="1"/>
     <row r="23" spans="1:8">
       <c r="A23" s="31" t="s">
         <v>5</v>
@@ -11735,8 +12871,12 @@
         <f>Tabla3[[#This Row],[Porcentaje de la muestra '[pct']]] *10000</f>
         <v>50</v>
       </c>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
+      <c r="C25" s="17">
+        <v>0.19</v>
+      </c>
+      <c r="D25" s="17">
+        <v>0.24</v>
+      </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="19">
@@ -11746,8 +12886,12 @@
         <f>Tabla3[[#This Row],[Porcentaje de la muestra '[pct']]] *10000</f>
         <v>500</v>
       </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
+      <c r="C26" s="4">
+        <v>4.53</v>
+      </c>
+      <c r="D26" s="4">
+        <v>2.72</v>
+      </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="18">
@@ -11757,8 +12901,12 @@
         <f>Tabla3[[#This Row],[Porcentaje de la muestra '[pct']]] *10000</f>
         <v>1000</v>
       </c>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
+      <c r="C27" s="17">
+        <v>11.75</v>
+      </c>
+      <c r="D27" s="17">
+        <v>5.83</v>
+      </c>
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="19">
@@ -11768,8 +12916,12 @@
         <f>Tabla3[[#This Row],[Porcentaje de la muestra '[pct']]] *10000</f>
         <v>2000</v>
       </c>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
+      <c r="C28" s="4">
+        <v>35.369999999999997</v>
+      </c>
+      <c r="D28" s="4">
+        <v>13.9</v>
+      </c>
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="18">
@@ -11779,8 +12931,12 @@
         <f>Tabla3[[#This Row],[Porcentaje de la muestra '[pct']]] *10000</f>
         <v>3000</v>
       </c>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
+      <c r="C29" s="17">
+        <v>72.02</v>
+      </c>
+      <c r="D29" s="17">
+        <v>20.46</v>
+      </c>
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="19">
@@ -11790,8 +12946,12 @@
         <f>Tabla3[[#This Row],[Porcentaje de la muestra '[pct']]] *10000</f>
         <v>5000</v>
       </c>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
+      <c r="C30" s="4">
+        <v>187.35</v>
+      </c>
+      <c r="D30" s="4">
+        <v>37.94</v>
+      </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="18">
@@ -11801,8 +12961,12 @@
         <f>Tabla3[[#This Row],[Porcentaje de la muestra '[pct']]] *10000</f>
         <v>8000</v>
       </c>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
+      <c r="C31" s="17">
+        <v>432.32</v>
+      </c>
+      <c r="D31" s="17">
+        <v>58.64</v>
+      </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="19">
@@ -11812,8 +12976,12 @@
         <f>Tabla3[[#This Row],[Porcentaje de la muestra '[pct']]] *10000</f>
         <v>10000</v>
       </c>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
+      <c r="C32" s="4">
+        <v>631.94000000000005</v>
+      </c>
+      <c r="D32" s="4">
+        <v>75.319999999999993</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -11841,119 +13009,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743">
-      <UserInfo>
-        <DisplayName>Carlos Andres Lozano Garzon</DisplayName>
-        <AccountId>13</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Dario Ernesto Correal Torres</DisplayName>
-        <AccountId>15</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Mario  Fernando De la rosa Rosero</DisplayName>
-        <AccountId>16</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Christian Camilo Aparicio Baquen</DisplayName>
-        <AccountId>50</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Arturo Henao Chaparro</DisplayName>
-        <AccountId>48</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Luis Esteban Florez Salamanca</DisplayName>
-        <AccountId>33</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Ivan David Salazar Cardenas</DisplayName>
-        <AccountId>52</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Juan Carlos Marin Morales</DisplayName>
-        <AccountId>53</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Sofia Duque Gomez</DisplayName>
-        <AccountId>60</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Andres Felipe Romero Brand</DisplayName>
-        <AccountId>91</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Lindsay Vanessa Pinto Morato</DisplayName>
-        <AccountId>92</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Miguel Angel Acosta Walteros</DisplayName>
-        <AccountId>94</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Juan David Diaz Ipuz</DisplayName>
-        <AccountId>90</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Lily Aitana valentina Duque Chavez</DisplayName>
-        <AccountId>17</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Isaac David Bermudez Lara</DisplayName>
-        <AccountId>95</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Daniel Alejandro Angel Fuertes</DisplayName>
-        <AccountId>55</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Jeniffer Liliam Mendoza Espinosa</DisplayName>
-        <AccountId>97</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Kevin Cohen Solano</DisplayName>
-        <AccountId>93</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Cesar Luis Moreno Gonzalez</DisplayName>
-        <AccountId>96</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Jose Cristobal Arroyo Castellanos</DisplayName>
-        <AccountId>54</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <TaxCatchAll xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="164883f8-7691-4ecf-b54a-664c0d0edefe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010023858CF01A2EF24688B692775F4C60A4" ma:contentTypeVersion="17" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="af74a0f8eb440a60883e9dd833f0742f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="164883f8-7691-4ecf-b54a-664c0d0edefe" xmlns:ns3="85e30bcc-d76c-4413-8e4d-2dce22fb0743" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f5ceeff32ffca1089660572a8ebd1782" ns2:_="" ns3:_="">
     <xsd:import namespace="164883f8-7691-4ecf-b54a-664c0d0edefe"/>
@@ -12202,6 +13257,119 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743">
+      <UserInfo>
+        <DisplayName>Carlos Andres Lozano Garzon</DisplayName>
+        <AccountId>13</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Dario Ernesto Correal Torres</DisplayName>
+        <AccountId>15</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Mario  Fernando De la rosa Rosero</DisplayName>
+        <AccountId>16</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Christian Camilo Aparicio Baquen</DisplayName>
+        <AccountId>50</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Arturo Henao Chaparro</DisplayName>
+        <AccountId>48</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Luis Esteban Florez Salamanca</DisplayName>
+        <AccountId>33</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Ivan David Salazar Cardenas</DisplayName>
+        <AccountId>52</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Juan Carlos Marin Morales</DisplayName>
+        <AccountId>53</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Sofia Duque Gomez</DisplayName>
+        <AccountId>60</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Andres Felipe Romero Brand</DisplayName>
+        <AccountId>91</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Lindsay Vanessa Pinto Morato</DisplayName>
+        <AccountId>92</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Miguel Angel Acosta Walteros</DisplayName>
+        <AccountId>94</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Juan David Diaz Ipuz</DisplayName>
+        <AccountId>90</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Lily Aitana valentina Duque Chavez</DisplayName>
+        <AccountId>17</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Isaac David Bermudez Lara</DisplayName>
+        <AccountId>95</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Daniel Alejandro Angel Fuertes</DisplayName>
+        <AccountId>55</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Jeniffer Liliam Mendoza Espinosa</DisplayName>
+        <AccountId>97</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Kevin Cohen Solano</DisplayName>
+        <AccountId>93</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Cesar Luis Moreno Gonzalez</DisplayName>
+        <AccountId>96</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Jose Cristobal Arroyo Castellanos</DisplayName>
+        <AccountId>54</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <TaxCatchAll xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="164883f8-7691-4ecf-b54a-664c0d0edefe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8DF3742-38F2-4B99-B335-CC4F04ED9F45}">
   <ds:schemaRefs>
@@ -12211,17 +13379,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C5E1E0-C817-4769-9D2D-1DC296B681FA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="85e30bcc-d76c-4413-8e4d-2dce22fb0743"/>
-    <ds:schemaRef ds:uri="164883f8-7691-4ecf-b54a-664c0d0edefe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24D72429-8592-4E2D-9A60-DFD77A3B0B84}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12238,4 +13395,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C5E1E0-C817-4769-9D2D-1DC296B681FA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="85e30bcc-d76c-4413-8e4d-2dce22fb0743"/>
+    <ds:schemaRef ds:uri="164883f8-7691-4ecf-b54a-664c0d0edefe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>